<commit_message>
Add project tracker exports and update README
</commit_message>
<xml_diff>
--- a/06-project-management/AI_Assisted_Release_Documentation_Workflow_Tracker.xlsx
+++ b/06-project-management/AI_Assisted_Release_Documentation_Workflow_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fafeff989e05c563/Career/Portfolio/ai-assisted-release-notes-workflow/06-project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="387" documentId="8_{24FF9882-0CC5-449F-AC87-0D2C8FBC8C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B878C73-5433-42BF-9BF2-3E311AB99629}"/>
+  <xr:revisionPtr revIDLastSave="397" documentId="8_{24FF9882-0CC5-449F-AC87-0D2C8FBC8C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{472B425A-C080-448A-AC18-1EB179A2F25A}"/>
   <bookViews>
-    <workbookView xWindow="-8250" yWindow="-20910" windowWidth="33010" windowHeight="20080" activeTab="1" xr2:uid="{DF2CF6FE-3307-4A0C-9333-6DB16CCCBAF2}"/>
+    <workbookView xWindow="-8910" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{DF2CF6FE-3307-4A0C-9333-6DB16CCCBAF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="398">
   <si>
     <t>WBS ID</t>
   </si>
@@ -1230,6 +1230,21 @@
   </si>
   <si>
     <t>Use the Validation Log to track issues such as truncated Mermaid labels, broken links, or unclear file references, and push changes to GitHub.</t>
+  </si>
+  <si>
+    <t>8.2R</t>
+  </si>
+  <si>
+    <t>Export project tracker tabs for GitHub viewing</t>
+  </si>
+  <si>
+    <t>Export key workbook tabs as Markdown or CSV so reviewers can inspect the project overview, WBS, decision log, prompt log, prompt run log, and validation log without opening Excel.</t>
+  </si>
+  <si>
+    <t>The Excel workbook remains the source tracker, but exported files make the project management evidence easier to view in GitHub.</t>
+  </si>
+  <si>
+    <t>Update README links to project management artefacts.</t>
   </si>
 </sst>
 </file>
@@ -1329,7 +1344,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="49">
+  <dxfs count="52">
     <dxf>
       <fill>
         <patternFill>
@@ -1373,6 +1388,27 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1430,37 +1466,37 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="20" formatCode="d\-mmm\-yy"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1534,94 +1570,94 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9C4856A4-1CA3-468C-9420-181B6923F3FD}" name="Table9" displayName="Table9" ref="A1:C23" totalsRowShown="0" headerRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9C4856A4-1CA3-468C-9420-181B6923F3FD}" name="Table9" displayName="Table9" ref="A1:C23" totalsRowShown="0" headerRowDxfId="41">
   <autoFilter ref="A1:C23" xr:uid="{9C4856A4-1CA3-468C-9420-181B6923F3FD}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{6FCC83BA-5C21-407C-89CC-B776018CFF77}" name="Section"/>
     <tableColumn id="2" xr3:uid="{385EC2F1-2375-4A15-B7F0-F7E0FEB03D9D}" name="Field"/>
-    <tableColumn id="3" xr3:uid="{036EEACA-41D8-45D3-A94A-64CFFD3406C1}" name="Details" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{036EEACA-41D8-45D3-A94A-64CFFD3406C1}" name="Details" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EFC9FEB-D1BA-4366-8993-849A0B92EC58}" name="Table1" displayName="Table1" ref="A1:H35" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
-  <autoFilter ref="A1:H35" xr:uid="{4EFC9FEB-D1BA-4366-8993-849A0B92EC58}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EFC9FEB-D1BA-4366-8993-849A0B92EC58}" name="Table1" displayName="Table1" ref="A1:H36" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+  <autoFilter ref="A1:H36" xr:uid="{4EFC9FEB-D1BA-4366-8993-849A0B92EC58}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5F51F6D7-E2D2-45BA-882E-706C10FFD150}" name="WBS ID" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{FA67913F-6181-4185-B8E2-001404C4F35C}" name="Phase" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{D3F3CB81-EBD1-467E-B985-4DD648E644ED}" name="Task Name" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{67E306BF-0C38-4579-8F51-156979593041}" name="Description" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{EB0314F5-D989-427C-ABAC-3C988732DA62}" name="Estimated Effort" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{E070EEC1-B75A-424F-931C-9D8F343CFE79}" name="Status" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{1793ADE6-8F3A-492C-BF02-9F0754A955AA}" name="Notes" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{34E05C4C-BEB9-46C3-B388-C2C1A5947DC3}" name="Next Action" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{5F51F6D7-E2D2-45BA-882E-706C10FFD150}" name="WBS ID" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{FA67913F-6181-4185-B8E2-001404C4F35C}" name="Phase" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{D3F3CB81-EBD1-467E-B985-4DD648E644ED}" name="Task Name" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{67E306BF-0C38-4579-8F51-156979593041}" name="Description" dataDxfId="46"/>
+    <tableColumn id="5" xr3:uid="{EB0314F5-D989-427C-ABAC-3C988732DA62}" name="Estimated Effort" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{E070EEC1-B75A-424F-931C-9D8F343CFE79}" name="Status" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{1793ADE6-8F3A-492C-BF02-9F0754A955AA}" name="Notes" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{34E05C4C-BEB9-46C3-B388-C2C1A5947DC3}" name="Next Action" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F925828B-3822-482F-AC33-1929821E1A13}" name="Table5" displayName="Table5" ref="A1:F7" totalsRowShown="0" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F925828B-3822-482F-AC33-1929821E1A13}" name="Table5" displayName="Table5" ref="A1:F7" totalsRowShown="0" dataDxfId="39">
   <autoFilter ref="A1:F7" xr:uid="{F925828B-3822-482F-AC33-1929821E1A13}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{8FC983B2-4C39-4D49-9083-2EBD8FFD5C73}" name="Decision ID"/>
-    <tableColumn id="2" xr3:uid="{3971E9A3-7B24-4402-B731-0FF018B03528}" name="Date" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{598FC76D-BCF7-4A23-A8CB-43F6DB24894D}" name="Decision" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{D2C64D8E-397A-4B88-99FD-5D836F0A2A62}" name="Context" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{0CED7B50-B0ED-453C-9461-EE66B27C8141}" name="Rationale" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{CE66CE7A-EBBF-4D45-992B-B662B2E4694B}" name="Impact / Action" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{3971E9A3-7B24-4402-B731-0FF018B03528}" name="Date" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{598FC76D-BCF7-4A23-A8CB-43F6DB24894D}" name="Decision" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{D2C64D8E-397A-4B88-99FD-5D836F0A2A62}" name="Context" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{0CED7B50-B0ED-453C-9461-EE66B27C8141}" name="Rationale" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{CE66CE7A-EBBF-4D45-992B-B662B2E4694B}" name="Impact / Action" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2F97A6A4-BE8C-4610-AB7A-27FE26948BCA}" name="Table1418" displayName="Table1418" ref="A1:H5" totalsRowShown="0" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2F97A6A4-BE8C-4610-AB7A-27FE26948BCA}" name="Table1418" displayName="Table1418" ref="A1:H5" totalsRowShown="0" dataDxfId="33">
   <autoFilter ref="A1:H5" xr:uid="{2F97A6A4-BE8C-4610-AB7A-27FE26948BCA}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{0B4CFDBB-B21A-4C79-9486-E49214581940}" name="Prompt ID"/>
     <tableColumn id="2" xr3:uid="{39EF02B1-2B06-492B-BA4E-CE33653F9A56}" name="Workflow Step"/>
-    <tableColumn id="3" xr3:uid="{2D06AFEC-F971-42C7-9EF2-DDCFF45A28F0}" name="Prompt Name" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{C4965871-1B4E-4606-A5B9-2A34A9389649}" name="Purpose" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{C962E6BF-9663-4F75-9C07-BDB1E74878E3}" name="Input Sources" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{D5353740-CE59-4D15-B5D0-C3D06E046F96}" name="Expected Output" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{43D28BC9-B2B0-4802-B742-55D820C3215C}" name="Status" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{CF0811A2-3202-4714-B186-3EFB1879C5D1}" name="Notes" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{2D06AFEC-F971-42C7-9EF2-DDCFF45A28F0}" name="Prompt Name" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{C4965871-1B4E-4606-A5B9-2A34A9389649}" name="Purpose" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{C962E6BF-9663-4F75-9C07-BDB1E74878E3}" name="Input Sources" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{D5353740-CE59-4D15-B5D0-C3D06E046F96}" name="Expected Output" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{43D28BC9-B2B0-4802-B742-55D820C3215C}" name="Status" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{CF0811A2-3202-4714-B186-3EFB1879C5D1}" name="Notes" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{12C51863-6E9D-4302-A30C-B368FC2ADBF2}" name="Table3" displayName="Table3" ref="A1:F5" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{12C51863-6E9D-4302-A30C-B368FC2ADBF2}" name="Table3" displayName="Table3" ref="A1:F5" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:F5" xr:uid="{12C51863-6E9D-4302-A30C-B368FC2ADBF2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{13ACCAA4-6950-4227-8494-727607E358D1}" name="Run ID" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{6F54ED06-FCFC-4A9A-A0E6-1BC139FB5DF6}" name="Prompt ID" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{136F677D-DF52-42B7-81C9-A0B839C6F461}" name="Input Sources" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{C77C704F-EC11-4AF1-9CB6-2FB47C08F98D}" name="Output Created" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{BCB089FF-4750-441F-B02C-6360F6B8E072}" name="Status" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{1F8D15B8-C303-4DDA-A84F-A6D335B503E0}" name="Notes" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{13ACCAA4-6950-4227-8494-727607E358D1}" name="Run ID" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{6F54ED06-FCFC-4A9A-A0E6-1BC139FB5DF6}" name="Prompt ID" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{136F677D-DF52-42B7-81C9-A0B839C6F461}" name="Input Sources" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{C77C704F-EC11-4AF1-9CB6-2FB47C08F98D}" name="Output Created" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{BCB089FF-4750-441F-B02C-6360F6B8E072}" name="Status" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{1F8D15B8-C303-4DDA-A84F-A6D335B503E0}" name="Notes" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{33A033F5-CCDE-4932-A411-A5E5A782CDE8}" name="Table6" displayName="Table6" ref="A1:I5" totalsRowShown="0" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{33A033F5-CCDE-4932-A411-A5E5A782CDE8}" name="Table6" displayName="Table6" ref="A1:I5" totalsRowShown="0" dataDxfId="18">
   <autoFilter ref="A1:I5" xr:uid="{33A033F5-CCDE-4932-A411-A5E5A782CDE8}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{2E3BF62F-34AD-4994-B572-7DBC9A972921}" name="Issue ID" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{5E5846B2-2BDB-496D-B1A0-C7FC54FB88BD}" name="Review Stage" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{8E0F951F-7D43-43F9-B90C-EFC81C855CA2}" name="File / Location" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{C07CC507-A444-4FCB-9B7C-DFCF8C64FFA3}" name="Issue Type" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{24E9DFDC-F5AF-4409-9BA2-D715DC193DE6}" name="Finding" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{47694A5B-0B4D-41BA-B01F-052E5F8DFEB4}" name="Severity" dataDxfId="42"/>
-    <tableColumn id="7" xr3:uid="{6822F15F-781B-4E57-A6CD-E7DC77537A1B}" name="Recommended Action" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{087035D6-532A-4291-A330-FEE9D8A6BBA4}" name="Status" dataDxfId="40"/>
-    <tableColumn id="9" xr3:uid="{604511E3-334B-4AE7-8191-A1BBF127313E}" name="Resolution Notes" dataDxfId="39"/>
+    <tableColumn id="1" xr3:uid="{2E3BF62F-34AD-4994-B572-7DBC9A972921}" name="Issue ID" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{5E5846B2-2BDB-496D-B1A0-C7FC54FB88BD}" name="Review Stage" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{8E0F951F-7D43-43F9-B90C-EFC81C855CA2}" name="File / Location" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{C07CC507-A444-4FCB-9B7C-DFCF8C64FFA3}" name="Issue Type" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{24E9DFDC-F5AF-4409-9BA2-D715DC193DE6}" name="Finding" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{47694A5B-0B4D-41BA-B01F-052E5F8DFEB4}" name="Severity" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{6822F15F-781B-4E57-A6CD-E7DC77537A1B}" name="Recommended Action" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{087035D6-532A-4291-A330-FEE9D8A6BBA4}" name="Status" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{604511E3-334B-4AE7-8191-A1BBF127313E}" name="Resolution Notes" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2387,7 +2423,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6301BFC-29FE-4EE3-A73C-DFE02EEBE774}">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.08984375" customWidth="1"/>
@@ -2999,174 +3035,174 @@
         <v>248</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>86</v>
+        <v>393</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>88</v>
+        <v>394</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>89</v>
+        <v>395</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>90</v>
+        <v>24</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>48</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>249</v>
+        <v>396</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>250</v>
+        <v>397</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>24</v>
+        <v>90</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>94</v>
+        <v>249</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>277</v>
+        <v>99</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>278</v>
+        <v>95</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>48</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>48</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>104</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>24</v>
@@ -3175,139 +3211,165 @@
         <v>48</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>295</v>
+        <v>282</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C31" t="s">
-        <v>296</v>
+      <c r="C31" s="1" t="s">
+        <v>111</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>48</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>314</v>
+        <v>294</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>315</v>
+        <v>113</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>316</v>
+      <c r="C32" t="s">
+        <v>296</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>317</v>
+        <v>114</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>392</v>
+        <v>314</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
-        <v>115</v>
+        <v>315</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>117</v>
+        <v>316</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>118</v>
+        <v>317</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>119</v>
+        <v>392</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>116</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>130</v>
+        <v>24</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G35" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="H36" s="1" t="s">
         <v>132</v>
       </c>
     </row>
@@ -3322,34 +3384,55 @@
       <c r="H39" s="1"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F1:F1048576">
-    <cfRule type="expression" dxfId="5" priority="31">
+    <cfRule type="expression" dxfId="8" priority="34">
       <formula>$F1="Draft complete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="32">
+    <cfRule type="expression" dxfId="7" priority="35">
       <formula>$F1="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="33">
+    <cfRule type="expression" dxfId="6" priority="36">
       <formula>$F1="Complete"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H38:H40">
-    <cfRule type="expression" dxfId="2" priority="37">
-      <formula>$H38="Draft complete"</formula>
+  <conditionalFormatting sqref="H39:H41">
+    <cfRule type="expression" dxfId="5" priority="40">
+      <formula>$H39="Draft complete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="38">
-      <formula>$H38="In progress"</formula>
+    <cfRule type="expression" dxfId="4" priority="41">
+      <formula>$H39="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="39">
-      <formula>$H38="Complete"</formula>
+    <cfRule type="expression" dxfId="3" priority="42">
+      <formula>$H39="Complete"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>$H24="Draft complete"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$H24="In progress"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>$H24="Complete"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Final polish for portfolio project
</commit_message>
<xml_diff>
--- a/06-project-management/AI_Assisted_Release_Documentation_Workflow_Tracker.xlsx
+++ b/06-project-management/AI_Assisted_Release_Documentation_Workflow_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fafeff989e05c563/Career/Portfolio/ai-assisted-release-notes-workflow/06-project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="397" documentId="8_{24FF9882-0CC5-449F-AC87-0D2C8FBC8C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{472B425A-C080-448A-AC18-1EB179A2F25A}"/>
+  <xr:revisionPtr revIDLastSave="429" documentId="8_{24FF9882-0CC5-449F-AC87-0D2C8FBC8C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB225FDF-53F5-4DB5-B3D4-B0893FBB12D1}"/>
   <bookViews>
     <workbookView xWindow="-8910" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{DF2CF6FE-3307-4A0C-9333-6DB16CCCBAF2}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="396">
   <si>
     <t>WBS ID</t>
   </si>
@@ -85,9 +85,6 @@
     <t>30 mins</t>
   </si>
   <si>
-    <t>Not started</t>
-  </si>
-  <si>
     <t>Reflects the new workflow where AI generates the release contents list from messy inputs.</t>
   </si>
   <si>
@@ -154,9 +151,6 @@
     <t>Keep P-000, P-003, P-004, and P-005. Archive P-001 and P-002 as baseline prompts.</t>
   </si>
   <si>
-    <t>In progress</t>
-  </si>
-  <si>
     <t>Prompt Log needs to match simplified workflow.</t>
   </si>
   <si>
@@ -403,12 +397,6 @@
     <t>Map revised project to high-velocity updates, AI workflow design, release triage, KB maintenance, and validation.</t>
   </si>
   <si>
-    <t>Useful for applications/interviews.</t>
-  </si>
-  <si>
-    <t>Create capability map.</t>
-  </si>
-  <si>
     <t>11.1R</t>
   </si>
   <si>
@@ -418,12 +406,6 @@
     <t>Write short description for portfolio, LinkedIn, or job applications.</t>
   </si>
   <si>
-    <t>Do after case study is stable.</t>
-  </si>
-  <si>
-    <t>Draft summary.</t>
-  </si>
-  <si>
     <t>12R</t>
   </si>
   <si>
@@ -437,9 +419,6 @@
   </si>
   <si>
     <t>1.5 hours</t>
-  </si>
-  <si>
-    <t>Final review after publication or local completion.</t>
   </si>
   <si>
     <t>Complete project.</t>
@@ -1229,9 +1208,6 @@
     <t>Reviewers can inspect the project planning without downloading anything, and the Excel workbook is still available as the original working artefact.</t>
   </si>
   <si>
-    <t>Use the Validation Log to track issues such as truncated Mermaid labels, broken links, or unclear file references, and push changes to GitHub.</t>
-  </si>
-  <si>
     <t>8.2R</t>
   </si>
   <si>
@@ -1245,6 +1221,24 @@
   </si>
   <si>
     <t>Update README links to project management artefacts.</t>
+  </si>
+  <si>
+    <t>GitHub repo review issues resolved and changes pushed.</t>
+  </si>
+  <si>
+    <t>Capability map created to connect the project evidence to release documentation, AI workflow design, KB planning, validation, docs-as-code awareness, and project management skills.</t>
+  </si>
+  <si>
+    <t>Write short portfolio summary.</t>
+  </si>
+  <si>
+    <t>Short project summary written for portfolio, GitHub README, or job application use.</t>
+  </si>
+  <si>
+    <t>Conduct final quality review.</t>
+  </si>
+  <si>
+    <t>Reviewing the GitHub repo, case study, README, links, diagrams, final outputs, and project management artefacts before treating the project as portfolio-ready.</t>
   </si>
 </sst>
 </file>
@@ -1344,28 +1338,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="52">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="49">
     <dxf>
       <fill>
         <patternFill>
@@ -1570,94 +1543,94 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9C4856A4-1CA3-468C-9420-181B6923F3FD}" name="Table9" displayName="Table9" ref="A1:C23" totalsRowShown="0" headerRowDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9C4856A4-1CA3-468C-9420-181B6923F3FD}" name="Table9" displayName="Table9" ref="A1:C23" totalsRowShown="0" headerRowDxfId="38">
   <autoFilter ref="A1:C23" xr:uid="{9C4856A4-1CA3-468C-9420-181B6923F3FD}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{6FCC83BA-5C21-407C-89CC-B776018CFF77}" name="Section"/>
     <tableColumn id="2" xr3:uid="{385EC2F1-2375-4A15-B7F0-F7E0FEB03D9D}" name="Field"/>
-    <tableColumn id="3" xr3:uid="{036EEACA-41D8-45D3-A94A-64CFFD3406C1}" name="Details" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{036EEACA-41D8-45D3-A94A-64CFFD3406C1}" name="Details" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EFC9FEB-D1BA-4366-8993-849A0B92EC58}" name="Table1" displayName="Table1" ref="A1:H36" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4EFC9FEB-D1BA-4366-8993-849A0B92EC58}" name="Table1" displayName="Table1" ref="A1:H36" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47">
   <autoFilter ref="A1:H36" xr:uid="{4EFC9FEB-D1BA-4366-8993-849A0B92EC58}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{5F51F6D7-E2D2-45BA-882E-706C10FFD150}" name="WBS ID" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{FA67913F-6181-4185-B8E2-001404C4F35C}" name="Phase" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{D3F3CB81-EBD1-467E-B985-4DD648E644ED}" name="Task Name" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{67E306BF-0C38-4579-8F51-156979593041}" name="Description" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{EB0314F5-D989-427C-ABAC-3C988732DA62}" name="Estimated Effort" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{E070EEC1-B75A-424F-931C-9D8F343CFE79}" name="Status" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{1793ADE6-8F3A-492C-BF02-9F0754A955AA}" name="Notes" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{34E05C4C-BEB9-46C3-B388-C2C1A5947DC3}" name="Next Action" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{5F51F6D7-E2D2-45BA-882E-706C10FFD150}" name="WBS ID" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{FA67913F-6181-4185-B8E2-001404C4F35C}" name="Phase" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{D3F3CB81-EBD1-467E-B985-4DD648E644ED}" name="Task Name" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{67E306BF-0C38-4579-8F51-156979593041}" name="Description" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{EB0314F5-D989-427C-ABAC-3C988732DA62}" name="Estimated Effort" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{E070EEC1-B75A-424F-931C-9D8F343CFE79}" name="Status" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{1793ADE6-8F3A-492C-BF02-9F0754A955AA}" name="Notes" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{34E05C4C-BEB9-46C3-B388-C2C1A5947DC3}" name="Next Action" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F925828B-3822-482F-AC33-1929821E1A13}" name="Table5" displayName="Table5" ref="A1:F7" totalsRowShown="0" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{F925828B-3822-482F-AC33-1929821E1A13}" name="Table5" displayName="Table5" ref="A1:F7" totalsRowShown="0" dataDxfId="36">
   <autoFilter ref="A1:F7" xr:uid="{F925828B-3822-482F-AC33-1929821E1A13}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{8FC983B2-4C39-4D49-9083-2EBD8FFD5C73}" name="Decision ID"/>
-    <tableColumn id="2" xr3:uid="{3971E9A3-7B24-4402-B731-0FF018B03528}" name="Date" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{598FC76D-BCF7-4A23-A8CB-43F6DB24894D}" name="Decision" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{D2C64D8E-397A-4B88-99FD-5D836F0A2A62}" name="Context" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{0CED7B50-B0ED-453C-9461-EE66B27C8141}" name="Rationale" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{CE66CE7A-EBBF-4D45-992B-B662B2E4694B}" name="Impact / Action" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{3971E9A3-7B24-4402-B731-0FF018B03528}" name="Date" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{598FC76D-BCF7-4A23-A8CB-43F6DB24894D}" name="Decision" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{D2C64D8E-397A-4B88-99FD-5D836F0A2A62}" name="Context" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{0CED7B50-B0ED-453C-9461-EE66B27C8141}" name="Rationale" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{CE66CE7A-EBBF-4D45-992B-B662B2E4694B}" name="Impact / Action" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2F97A6A4-BE8C-4610-AB7A-27FE26948BCA}" name="Table1418" displayName="Table1418" ref="A1:H5" totalsRowShown="0" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2F97A6A4-BE8C-4610-AB7A-27FE26948BCA}" name="Table1418" displayName="Table1418" ref="A1:H5" totalsRowShown="0" dataDxfId="30">
   <autoFilter ref="A1:H5" xr:uid="{2F97A6A4-BE8C-4610-AB7A-27FE26948BCA}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{0B4CFDBB-B21A-4C79-9486-E49214581940}" name="Prompt ID"/>
     <tableColumn id="2" xr3:uid="{39EF02B1-2B06-492B-BA4E-CE33653F9A56}" name="Workflow Step"/>
-    <tableColumn id="3" xr3:uid="{2D06AFEC-F971-42C7-9EF2-DDCFF45A28F0}" name="Prompt Name" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{C4965871-1B4E-4606-A5B9-2A34A9389649}" name="Purpose" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{C962E6BF-9663-4F75-9C07-BDB1E74878E3}" name="Input Sources" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{D5353740-CE59-4D15-B5D0-C3D06E046F96}" name="Expected Output" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{43D28BC9-B2B0-4802-B742-55D820C3215C}" name="Status" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{CF0811A2-3202-4714-B186-3EFB1879C5D1}" name="Notes" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{2D06AFEC-F971-42C7-9EF2-DDCFF45A28F0}" name="Prompt Name" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{C4965871-1B4E-4606-A5B9-2A34A9389649}" name="Purpose" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{C962E6BF-9663-4F75-9C07-BDB1E74878E3}" name="Input Sources" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{D5353740-CE59-4D15-B5D0-C3D06E046F96}" name="Expected Output" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{43D28BC9-B2B0-4802-B742-55D820C3215C}" name="Status" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{CF0811A2-3202-4714-B186-3EFB1879C5D1}" name="Notes" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{12C51863-6E9D-4302-A30C-B368FC2ADBF2}" name="Table3" displayName="Table3" ref="A1:F5" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{12C51863-6E9D-4302-A30C-B368FC2ADBF2}" name="Table3" displayName="Table3" ref="A1:F5" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:F5" xr:uid="{12C51863-6E9D-4302-A30C-B368FC2ADBF2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{13ACCAA4-6950-4227-8494-727607E358D1}" name="Run ID" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{6F54ED06-FCFC-4A9A-A0E6-1BC139FB5DF6}" name="Prompt ID" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{136F677D-DF52-42B7-81C9-A0B839C6F461}" name="Input Sources" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{C77C704F-EC11-4AF1-9CB6-2FB47C08F98D}" name="Output Created" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{BCB089FF-4750-441F-B02C-6360F6B8E072}" name="Status" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{1F8D15B8-C303-4DDA-A84F-A6D335B503E0}" name="Notes" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{13ACCAA4-6950-4227-8494-727607E358D1}" name="Run ID" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{6F54ED06-FCFC-4A9A-A0E6-1BC139FB5DF6}" name="Prompt ID" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{136F677D-DF52-42B7-81C9-A0B839C6F461}" name="Input Sources" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{C77C704F-EC11-4AF1-9CB6-2FB47C08F98D}" name="Output Created" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{BCB089FF-4750-441F-B02C-6360F6B8E072}" name="Status" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{1F8D15B8-C303-4DDA-A84F-A6D335B503E0}" name="Notes" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{33A033F5-CCDE-4932-A411-A5E5A782CDE8}" name="Table6" displayName="Table6" ref="A1:I5" totalsRowShown="0" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{33A033F5-CCDE-4932-A411-A5E5A782CDE8}" name="Table6" displayName="Table6" ref="A1:I5" totalsRowShown="0" dataDxfId="15">
   <autoFilter ref="A1:I5" xr:uid="{33A033F5-CCDE-4932-A411-A5E5A782CDE8}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{2E3BF62F-34AD-4994-B572-7DBC9A972921}" name="Issue ID" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{5E5846B2-2BDB-496D-B1A0-C7FC54FB88BD}" name="Review Stage" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{8E0F951F-7D43-43F9-B90C-EFC81C855CA2}" name="File / Location" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{C07CC507-A444-4FCB-9B7C-DFCF8C64FFA3}" name="Issue Type" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{24E9DFDC-F5AF-4409-9BA2-D715DC193DE6}" name="Finding" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{47694A5B-0B4D-41BA-B01F-052E5F8DFEB4}" name="Severity" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{6822F15F-781B-4E57-A6CD-E7DC77537A1B}" name="Recommended Action" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{087035D6-532A-4291-A330-FEE9D8A6BBA4}" name="Status" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{604511E3-334B-4AE7-8191-A1BBF127313E}" name="Resolution Notes" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{2E3BF62F-34AD-4994-B572-7DBC9A972921}" name="Issue ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{5E5846B2-2BDB-496D-B1A0-C7FC54FB88BD}" name="Review Stage" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{8E0F951F-7D43-43F9-B90C-EFC81C855CA2}" name="File / Location" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{C07CC507-A444-4FCB-9B7C-DFCF8C64FFA3}" name="Issue Type" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{24E9DFDC-F5AF-4409-9BA2-D715DC193DE6}" name="Finding" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{47694A5B-0B4D-41BA-B01F-052E5F8DFEB4}" name="Severity" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{6822F15F-781B-4E57-A6CD-E7DC77537A1B}" name="Recommended Action" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{087035D6-532A-4291-A330-FEE9D8A6BBA4}" name="Status" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{604511E3-334B-4AE7-8191-A1BBF127313E}" name="Resolution Notes" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1996,22 +1969,22 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>5</v>
@@ -2019,344 +1992,344 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="J2" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B3" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="5"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>145</v>
-      </c>
       <c r="H4" s="5" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B5" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B6" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>383</v>
+        <v>376</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B7" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B8" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="44" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="B9" t="s">
-        <v>160</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>161</v>
       </c>
       <c r="J9" s="10"/>
     </row>
     <row r="10" spans="1:11" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B10" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B11" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B12" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B13" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>158</v>
+      </c>
+      <c r="B14" t="s">
         <v>165</v>
       </c>
-      <c r="B14" t="s">
-        <v>172</v>
-      </c>
       <c r="C14" s="1" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B15" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>168</v>
+      </c>
+      <c r="B16" t="s">
+        <v>173</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B16" t="s">
-        <v>180</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="H16" s="4" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B17" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B18" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B19" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B20" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B21" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="B22" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="B23" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B26" s="8">
         <v>46173</v>
       </c>
       <c r="C26" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="B27" s="8">
         <v>46177</v>
       </c>
       <c r="C27" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B28" s="8">
         <v>46178</v>
@@ -2451,7 +2424,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
@@ -2480,897 +2453,897 @@
         <v>12</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>336</v>
-      </c>
       <c r="H7" s="1" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="E13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="E15" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="E16" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="E17" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="E18" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="F19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="H19" t="s">
         <v>69</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="H19" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" s="1" t="s">
+      <c r="E20" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="H20" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>78</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="H21" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="E22" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="H22" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="E23" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="H23" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="E25" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>90</v>
-      </c>
       <c r="F25" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="E26" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G26" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="H26" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="E28" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>106</v>
-      </c>
       <c r="E29" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="E30" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="E31" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C32" t="s">
+        <v>289</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C32" t="s">
-        <v>296</v>
-      </c>
-      <c r="D32" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G32" s="1" t="s">
-        <v>314</v>
-      </c>
-      <c r="H32" s="1" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
-        <v>315</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G33" s="1" t="s">
+      <c r="C34" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="H34" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="H33" s="1" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C34" s="1" t="s">
+    </row>
+    <row r="35" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="B35" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="E35" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C35" s="1" t="s">
+      <c r="C36" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="D36" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" s="1" t="s">
+      <c r="E36" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="F36" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="H36" s="1" t="s">
         <v>125</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A36" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
@@ -3378,8 +3351,6 @@
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
     </row>
@@ -3388,8 +3359,6 @@
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
     </row>
@@ -3402,29 +3371,18 @@
       <c r="F42" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F1:F1048576">
-    <cfRule type="expression" dxfId="8" priority="34">
+  <conditionalFormatting sqref="F1:F38 F41:F1048576">
+    <cfRule type="expression" dxfId="5" priority="34">
       <formula>$F1="Draft complete"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="35">
+    <cfRule type="expression" dxfId="4" priority="35">
       <formula>$F1="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="36">
+    <cfRule type="expression" dxfId="3" priority="36">
       <formula>$F1="Complete"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H39:H41">
-    <cfRule type="expression" dxfId="5" priority="40">
-      <formula>$H39="Draft complete"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="41">
-      <formula>$H39="In progress"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="42">
-      <formula>$H39="Complete"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H24">
+  <conditionalFormatting sqref="H24 H41">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>$H24="Draft complete"</formula>
     </cfRule>
@@ -3455,144 +3413,144 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="B1" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C1" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="D1" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E1" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="F1" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="145" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="B2" s="8">
         <v>46177</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="B3" s="8">
         <v>46178</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="B4" s="8">
         <v>46178</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="B5" s="8">
         <v>46178</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="B6" s="8">
         <v>46178</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="B7" s="8">
         <v>46178</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
     </row>
   </sheetData>
@@ -3617,22 +3575,22 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B1" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="C1" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="D1" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="E1" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="F1" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
@@ -3643,106 +3601,106 @@
     </row>
     <row r="2" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="B2" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="B4" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B5" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3765,16 +3723,16 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
@@ -3785,82 +3743,82 @@
     </row>
     <row r="2" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -3888,112 +3846,112 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="B1" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="C1" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="D1" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="E1" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="F1" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="G1" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="H1" t="s">
         <v>5</v>
       </c>
       <c r="I1" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>306</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>309</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">

</xml_diff>